<commit_message>
phase-1: audit boundaries and establish architecture
</commit_message>
<xml_diff>
--- a/data/reconciliation_results.xlsx
+++ b/data/reconciliation_results.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>AI Confirmed: Matching order ID, date, and amount</t>
+          <t>AI Confirmed: Matching amount, date, and narration text</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Matching order ID, date, and amount</t>
+          <t>Matching amount, date, and narration text</t>
         </is>
       </c>
       <c r="J57" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>AI Confirmed: The transaction details from the ledger match the bank candidate provided, with a fee deduction correctly accounted for.</t>
+          <t>AI Confirmed: The transaction details match the bank candidate provided, with consistent amount, date, and explanatory narration.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>The transaction details from the ledger match the bank candidate provided, with a fee deduction correctly accounted for.</t>
+          <t>The transaction details match the bank candidate provided, with consistent amount, date, and explanatory narration.</t>
         </is>
       </c>
       <c r="J58" t="n">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>AI Confirmed: The transaction details match with a fee deduction.</t>
+          <t>AI Confirmed: All key attributes align: reference ID, amount (including fee), and date match, and the deterministic score (0.76) supports the match.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>The transaction details match with a fee deduction.</t>
+          <t>All key attributes align: reference ID, amount (including fee), and date match, and the deterministic score (0.76) supports the match.</t>
         </is>
       </c>
       <c r="J59" t="n">
@@ -3046,12 +3046,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>MATCHED</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>AI_CONFIRMED_MATCH</t>
+          <t>AI_REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -3059,7 +3059,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>AI Confirmed: Transaction reference, amount (including fee deduction), and dates all align between the ledger and the bank candidate.</t>
+          <t>AI Review: AI error: Request timed out.. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Transaction reference, amount (including fee deduction), and dates all align between the ledger and the bank candidate.</t>
+          <t>AI error: Request timed out.. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J60" t="n">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>AI Confirmed: Transaction details match ledger information</t>
+          <t>AI Confirmed: The transaction details match: the ledger amount equals the bank candidate's credited amount plus the deducted fee, and the dates align.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3122,7 +3122,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Transaction details match ledger information</t>
+          <t>The transaction details match: the ledger amount equals the bank candidate's credited amount plus the deducted fee, and the dates align.</t>
         </is>
       </c>
       <c r="J61" t="n">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>AI Confirmed: The transaction details in the ledger match the bank candidate, with the deduction fee accounting for the difference in amounts.</t>
+          <t>AI Confirmed: All key attributes (reference, amount, date) align; fee accounted for</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>The transaction details in the ledger match the bank candidate, with the deduction fee accounting for the difference in amounts.</t>
+          <t>All key attributes (reference, amount, date) align; fee accounted for</t>
         </is>
       </c>
       <c r="J62" t="n">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>AI Confirmed: All critical fields match (order ID, amount after accounting for fee, date, currency) and the deterministic score (0.7756) is high, indicating this bank entry corresponds to the ledger transaction.</t>
+          <t>AI Confirmed: The transaction details are consistent with a minor adjustment for a deduction fee.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>All critical fields match (order ID, amount after accounting for fee, date, currency) and the deterministic score (0.7756) is high, indicating this bank entry corresponds to the ledger transaction.</t>
+          <t>The transaction details are consistent with a minor adjustment for a deduction fee.</t>
         </is>
       </c>
       <c r="J63" t="n">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>AI Confirmed: Transaction details match</t>
+          <t>AI Confirmed: All key attributes match: the order ID is referenced in the narration, the amounts align after accounting for the fee, and the dates are identical, indicating the ledger transaction corresponds to this bank entry.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Transaction details match</t>
+          <t>All key attributes match: the order ID is referenced in the narration, the amounts align after accounting for the fee, and the dates are identical, indicating the ledger transaction corresponds to this bank entry.</t>
         </is>
       </c>
       <c r="J64" t="n">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>AI Confirmed: All transaction details match, including amount, date, reference, and fee consistency.</t>
+          <t>AI Confirmed: Transaction details align (order ID, date, and fee) despite the credited amount being lower due to the documented fee</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>All transaction details match, including amount, date, reference, and fee consistency.</t>
+          <t>Transaction details align (order ID, date, and fee) despite the credited amount being lower due to the documented fee</t>
         </is>
       </c>
       <c r="J65" t="n">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>AI Confirmed: The transaction details match: same date, correct amount difference as fee.</t>
+          <t>AI Confirmed: Order ID matches and fee deduction explains amount difference, so this is the correct transaction.</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>The transaction details match: same date, correct amount difference as fee.</t>
+          <t>Order ID matches and fee deduction explains amount difference, so this is the correct transaction.</t>
         </is>
       </c>
       <c r="J66" t="n">
@@ -3382,12 +3382,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHED</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>AI_CONFIRMED_MATCH</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Request timed out.. Safe fallback to REVIEW.</t>
+          <t>AI Confirmed: Exact match of amount, date, and relevant narration with ledger entry</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>AI error: Request timed out.. Safe fallback to REVIEW.</t>
+          <t>Exact match of amount, date, and relevant narration with ledger entry</t>
         </is>
       </c>
       <c r="J67" t="n">
@@ -3430,12 +3430,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>MATCHED</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>AI_CONFIRMED_MATCH</t>
+          <t>AI_REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>AI Confirmed: Transaction details match with bank candidate</t>
+          <t>AI Review: AI error: Request timed out.. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Transaction details match with bank candidate</t>
+          <t>AI error: Request timed out.. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J68" t="n">
@@ -3478,12 +3478,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHED</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>AI_CONFIRMED_MATCH</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>AI Review: Amount and date match between ledger and bank record, but the reference evidence (order ID) is not present in the narration, so the transaction cannot be confirmed as the same.</t>
+          <t>AI Confirmed: Transaction details are consistent</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Amount and date match between ledger and bank record, but the reference evidence (order ID) is not present in the narration, so the transaction cannot be confirmed as the same.</t>
+          <t>Transaction details are consistent</t>
         </is>
       </c>
       <c r="J69" t="n">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>AI Confirmed: Matching amount, date, and reference</t>
+          <t>AI Confirmed: Matching amount, date, and reference evidence</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Matching amount, date, and reference</t>
+          <t>Matching amount, date, and reference evidence</t>
         </is>
       </c>
       <c r="J70" t="n">
@@ -3574,12 +3574,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHED</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>AI_CONFIRMED_MATCH</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI Confirmed: Transaction details match</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>Transaction details match</t>
         </is>
       </c>
       <c r="J71" t="n">
@@ -3943,15 +3943,15 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>LOW_SCORE</t>
+          <t>NO_CANDIDATE</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>0.34</v>
+        <v>0</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Top score (0.34) below review threshold</t>
+          <t>No candidate within broad window and tolerance</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="n">
-        <v>0.34</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -4022,12 +4022,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHED</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>AI_CONFIRMED_MATCH</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -4035,7 +4035,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI Confirmed: Candidate 1 matches the ledger details perfectly</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>Candidate 1 matches the ledger details perfectly</t>
         </is>
       </c>
       <c r="J82" t="n">
@@ -4065,17 +4065,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>UTR500081</t>
+          <t>UTR500082</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHED</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>AI_CONFIRMED_MATCH</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI Confirmed: Strong match based on amount, date, and narration</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>Strong match based on amount, date, and narration</t>
         </is>
       </c>
       <c r="J83" t="n">
@@ -4118,12 +4118,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHED</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>AI_CONFIRMED_MATCH</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI Confirmed: Matching transaction details</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>Matching transaction details</t>
         </is>
       </c>
       <c r="J84" t="n">
@@ -4161,17 +4161,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>UTR500083</t>
+          <t>UTR500084</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHED</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>AI_CONFIRMED_MATCH</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI Confirmed: Matching amount, date, and narration text</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>Matching amount, date, and narration text</t>
         </is>
       </c>
       <c r="J85" t="n">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>UTR500083</t>
+          <t>UTR500085</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI Review: Both candidates have identical amount, date, and score, making it ambiguous which UTR matches the ledger entry</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>Both candidates have identical amount, date, and score, making it ambiguous which UTR matches the ledger entry</t>
         </is>
       </c>
       <c r="J86" t="n">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>UTR500083</t>
+          <t>UTR500085</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on tokens per minute (TPM): Limit 30000, Used 28478, Requested 2244. Please try again in 1.444s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per minute (RPM): Limit 30, Used 30, Requested 1. Please try again in 2s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `meta-llama/llama-4-scout-17b-16e-instruct` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on tokens per minute (TPM): Limit 30000, Used 28478, Requested 2244. Please try again in 1.444s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'compound', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J87" t="n">
@@ -4861,7 +4861,7 @@
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="inlineStr">
         <is>
-          <t>UTR500082</t>
+          <t>UTR500086</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4901,7 +4901,7 @@
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="inlineStr">
         <is>
-          <t>UTR500084</t>
+          <t>UTR500087</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4941,7 +4941,7 @@
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="inlineStr">
         <is>
-          <t>UTR500085</t>
+          <t>UTR500088</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4974,126 +4974,6 @@
       </c>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr"/>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>UTR500086</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>UNMATCHED</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>NO_MATCH</t>
-        </is>
-      </c>
-      <c r="E105" t="n">
-        <v>0</v>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>No matching ledger record found</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>deterministic</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr"/>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>UTR500087</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>UNMATCHED</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>NO_MATCH</t>
-        </is>
-      </c>
-      <c r="E106" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>No matching ledger record found</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>deterministic</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr"/>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>UTR500088</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>UNMATCHED</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>NO_MATCH</t>
-        </is>
-      </c>
-      <c r="E107" t="n">
-        <v>0</v>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>No matching ledger record found</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>deterministic</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5185,47 +5065,47 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C2" t="n">
         <v>21</v>
       </c>
       <c r="D2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G2" t="n">
         <v>55</v>
       </c>
       <c r="H2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="K2" t="n">
-        <v>0.8209</v>
+        <v>0.7639</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9016</v>
+        <v>0.8661</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>[{'order_id': 'ORD-1036', 'bank_id': 'UTR500036', 'scenario': 'fee_difference', 'ai_reason': 'Matching order ID, date, and amount', 'model': 'groq/compound', 'final_decision': 'MATCHED', 'orig_score': 0.7516}, {'order_id': 'ORD-1037', 'bank_id': 'UTR500037', 'scenario': 'fee_difference', 'ai_reason': 'The transaction details from the ledger match the bank candidate provided, with a fee deduction correctly accounted for.', 'model': 'groq/compound', 'final_decision': 'MATCHED', 'orig_score': 0.7756}, {'order_id': 'ORD-1038', 'bank_id': 'UTR500038', 'scenario': 'fee_difference', 'ai_reason': 'The transaction details match with a fee deduction.', 'model': 'groq/compound', 'final_decision': 'MATCHED', 'orig_score': 0.76}]</t>
+          <t>[{'order_id': 'ORD-1036', 'bank_id': 'UTR500036', 'scenario': 'fee_difference', 'ai_reason': 'Matching amount, date, and narration text', 'model': 'groq/compound', 'final_decision': 'MATCHED', 'orig_score': 0.7516}, {'order_id': 'ORD-1037', 'bank_id': 'UTR500037', 'scenario': 'fee_difference', 'ai_reason': 'The transaction details match the bank candidate provided, with consistent amount, date, and explanatory narration.', 'model': 'groq/compound', 'final_decision': 'MATCHED', 'orig_score': 0.7756}, {'order_id': 'ORD-1038', 'bank_id': 'UTR500038', 'scenario': 'fee_difference', 'ai_reason': 'All key attributes align: reference ID, amount (including fee), and date match, and the deterministic score (0.76) supports the match.', 'model': 'groq/compound', 'final_decision': 'MATCHED', 'orig_score': 0.76}]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
phase-4: finalize audit docs tests and judge demo
</commit_message>
<xml_diff>
--- a/data/reconciliation_results.xlsx
+++ b/data/reconciliation_results.xlsx
@@ -9823,7 +9823,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -9833,12 +9833,12 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J168" t="n">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -9893,12 +9893,12 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J169" t="n">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -9953,12 +9953,12 @@
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J170" t="n">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -10013,12 +10013,12 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J171" t="n">
@@ -10063,7 +10063,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -10073,12 +10073,12 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J172" t="n">
@@ -10123,7 +10123,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -10133,12 +10133,12 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J173" t="n">
@@ -10183,7 +10183,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -10193,12 +10193,12 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J174" t="n">
@@ -10243,7 +10243,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -10253,12 +10253,12 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J175" t="n">
@@ -10303,7 +10303,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -10313,12 +10313,12 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J176" t="n">
@@ -10363,7 +10363,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -10373,12 +10373,12 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J177" t="n">
@@ -10423,7 +10423,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -10433,12 +10433,12 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J178" t="n">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -10493,12 +10493,12 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J179" t="n">
@@ -10543,7 +10543,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -10553,12 +10553,12 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J180" t="n">
@@ -10603,7 +10603,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -10613,12 +10613,12 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J181" t="n">
@@ -10663,7 +10663,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -10673,12 +10673,12 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J182" t="n">
@@ -10723,7 +10723,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -10733,12 +10733,12 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J183" t="n">
@@ -10783,7 +10783,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -10793,12 +10793,12 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J184" t="n">
@@ -10843,7 +10843,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -10853,12 +10853,12 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J185" t="n">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -10913,12 +10913,12 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J186" t="n">
@@ -10963,7 +10963,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -10973,12 +10973,12 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J187" t="n">
@@ -11023,7 +11023,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -11033,12 +11033,12 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J188" t="n">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -11093,12 +11093,12 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J189" t="n">
@@ -11143,7 +11143,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -11153,12 +11153,12 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J190" t="n">
@@ -11203,7 +11203,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -11213,12 +11213,12 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J191" t="n">
@@ -11263,7 +11263,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -11273,12 +11273,12 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J192" t="n">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -11333,12 +11333,12 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J193" t="n">
@@ -11383,7 +11383,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -11393,12 +11393,12 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J194" t="n">
@@ -11443,7 +11443,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -11453,12 +11453,12 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J195" t="n">
@@ -11503,7 +11503,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -11513,12 +11513,12 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J196" t="n">
@@ -11563,7 +11563,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -11573,12 +11573,12 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J197" t="n">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -11633,12 +11633,12 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J198" t="n">
@@ -11683,7 +11683,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -11693,12 +11693,12 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J199" t="n">
@@ -11743,7 +11743,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -11753,12 +11753,12 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J200" t="n">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -11813,12 +11813,12 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J201" t="n">
@@ -11863,7 +11863,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -11873,12 +11873,12 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J202" t="n">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -11933,12 +11933,12 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J203" t="n">
@@ -11983,7 +11983,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -11993,12 +11993,12 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J204" t="n">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -12053,12 +12053,12 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J205" t="n">
@@ -12103,7 +12103,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -12113,12 +12113,12 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J206" t="n">
@@ -12163,7 +12163,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -12173,12 +12173,12 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J207" t="n">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -12233,12 +12233,12 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J208" t="n">
@@ -12283,7 +12283,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
@@ -12293,12 +12293,12 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J209" t="n">
@@ -12343,7 +12343,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
@@ -12353,12 +12353,12 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J210" t="n">
@@ -12403,7 +12403,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -12413,12 +12413,12 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J211" t="n">
@@ -12463,7 +12463,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -12473,12 +12473,12 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J212" t="n">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
@@ -12585,12 +12585,12 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J214" t="n">
@@ -12895,7 +12895,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -12905,12 +12905,12 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J220" t="n">
@@ -12955,7 +12955,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -12965,12 +12965,12 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J221" t="n">
@@ -13067,7 +13067,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -13077,12 +13077,12 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J223" t="n">
@@ -13127,7 +13127,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -13137,12 +13137,12 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J224" t="n">
@@ -13187,7 +13187,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -13197,12 +13197,12 @@
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J225" t="n">
@@ -13247,7 +13247,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>AI Review: Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -13257,12 +13257,12 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>groq/compound</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>Failed to initialize Groq client: No module named 'groq'</t>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="J226" t="n">

</xml_diff>

<commit_message>
phase-final: harden reconciliation benchmark api and debug flow
</commit_message>
<xml_diff>
--- a/data/reconciliation_results.xlsx
+++ b/data/reconciliation_results.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N259"/>
+  <dimension ref="A1:N260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4524,7 +4524,7 @@
         <v>0</v>
       </c>
       <c r="L73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M73" t="n">
         <v>1</v>
@@ -4692,7 +4692,7 @@
         <v>0</v>
       </c>
       <c r="L76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M76" t="n">
         <v>1</v>
@@ -4748,7 +4748,7 @@
         <v>0</v>
       </c>
       <c r="L77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M77" t="n">
         <v>1</v>
@@ -4804,7 +4804,7 @@
         <v>0</v>
       </c>
       <c r="L78" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M78" t="n">
         <v>1</v>
@@ -4860,7 +4860,7 @@
         <v>0</v>
       </c>
       <c r="L79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M79" t="n">
         <v>1</v>
@@ -5084,7 +5084,7 @@
         <v>0</v>
       </c>
       <c r="L83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M83" t="n">
         <v>1</v>
@@ -5140,7 +5140,7 @@
         <v>0</v>
       </c>
       <c r="L84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M84" t="n">
         <v>1</v>
@@ -5196,7 +5196,7 @@
         <v>0</v>
       </c>
       <c r="L85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M85" t="n">
         <v>1</v>
@@ -5252,7 +5252,7 @@
         <v>0</v>
       </c>
       <c r="L86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M86" t="n">
         <v>1</v>
@@ -5308,7 +5308,7 @@
         <v>0</v>
       </c>
       <c r="L87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M87" t="n">
         <v>1</v>
@@ -5420,7 +5420,7 @@
         <v>0</v>
       </c>
       <c r="L89" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M89" t="n">
         <v>1</v>
@@ -5476,7 +5476,7 @@
         <v>0</v>
       </c>
       <c r="L90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M90" t="n">
         <v>1</v>
@@ -5532,7 +5532,7 @@
         <v>0</v>
       </c>
       <c r="L91" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M91" t="n">
         <v>1</v>
@@ -9845,7 +9845,7 @@
         <v>0.72</v>
       </c>
       <c r="K168" t="n">
-        <v>49.06</v>
+        <v>48.91</v>
       </c>
       <c r="L168" t="n">
         <v>0</v>
@@ -9854,7 +9854,7 @@
         <v>1</v>
       </c>
       <c r="N168" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="169">
@@ -9905,7 +9905,7 @@
         <v>0.72</v>
       </c>
       <c r="K169" t="n">
-        <v>15.21</v>
+        <v>43.89</v>
       </c>
       <c r="L169" t="n">
         <v>0</v>
@@ -9914,7 +9914,7 @@
         <v>1</v>
       </c>
       <c r="N169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="170">
@@ -9965,7 +9965,7 @@
         <v>0.72</v>
       </c>
       <c r="K170" t="n">
-        <v>21.57</v>
+        <v>40.89</v>
       </c>
       <c r="L170" t="n">
         <v>0</v>
@@ -9974,7 +9974,7 @@
         <v>1</v>
       </c>
       <c r="N170" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="171">
@@ -10025,7 +10025,7 @@
         <v>0.72</v>
       </c>
       <c r="K171" t="n">
-        <v>42.02</v>
+        <v>11.18</v>
       </c>
       <c r="L171" t="n">
         <v>0</v>
@@ -10034,7 +10034,7 @@
         <v>1</v>
       </c>
       <c r="N171" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172">
@@ -10085,7 +10085,7 @@
         <v>0.72</v>
       </c>
       <c r="K172" t="n">
-        <v>21.77</v>
+        <v>11.14</v>
       </c>
       <c r="L172" t="n">
         <v>0</v>
@@ -10094,7 +10094,7 @@
         <v>1</v>
       </c>
       <c r="N172" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="173">
@@ -10145,7 +10145,7 @@
         <v>0.72</v>
       </c>
       <c r="K173" t="n">
-        <v>23.03</v>
+        <v>38.18</v>
       </c>
       <c r="L173" t="n">
         <v>0</v>
@@ -10154,7 +10154,7 @@
         <v>1</v>
       </c>
       <c r="N173" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="174">
@@ -10205,7 +10205,7 @@
         <v>0.72</v>
       </c>
       <c r="K174" t="n">
-        <v>39.82</v>
+        <v>24.72</v>
       </c>
       <c r="L174" t="n">
         <v>0</v>
@@ -10214,7 +10214,7 @@
         <v>1</v>
       </c>
       <c r="N174" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
@@ -10265,7 +10265,7 @@
         <v>0.72</v>
       </c>
       <c r="K175" t="n">
-        <v>12.82</v>
+        <v>34.4</v>
       </c>
       <c r="L175" t="n">
         <v>0</v>
@@ -10274,7 +10274,7 @@
         <v>1</v>
       </c>
       <c r="N175" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="176">
@@ -10325,7 +10325,7 @@
         <v>0.72</v>
       </c>
       <c r="K176" t="n">
-        <v>41.12</v>
+        <v>29.38</v>
       </c>
       <c r="L176" t="n">
         <v>0</v>
@@ -10385,7 +10385,7 @@
         <v>0.72</v>
       </c>
       <c r="K177" t="n">
-        <v>49.32</v>
+        <v>22.06</v>
       </c>
       <c r="L177" t="n">
         <v>0</v>
@@ -10394,7 +10394,7 @@
         <v>1</v>
       </c>
       <c r="N177" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="178">
@@ -10445,7 +10445,7 @@
         <v>0.72</v>
       </c>
       <c r="K178" t="n">
-        <v>39.15</v>
+        <v>29.95</v>
       </c>
       <c r="L178" t="n">
         <v>0</v>
@@ -10505,7 +10505,7 @@
         <v>0.72</v>
       </c>
       <c r="K179" t="n">
-        <v>17.36</v>
+        <v>24.35</v>
       </c>
       <c r="L179" t="n">
         <v>0</v>
@@ -10514,7 +10514,7 @@
         <v>1</v>
       </c>
       <c r="N179" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="180">
@@ -10565,7 +10565,7 @@
         <v>0.72</v>
       </c>
       <c r="K180" t="n">
-        <v>20.82</v>
+        <v>12.76</v>
       </c>
       <c r="L180" t="n">
         <v>0</v>
@@ -10625,7 +10625,7 @@
         <v>0.72</v>
       </c>
       <c r="K181" t="n">
-        <v>20.19</v>
+        <v>22.48</v>
       </c>
       <c r="L181" t="n">
         <v>0</v>
@@ -10634,7 +10634,7 @@
         <v>1</v>
       </c>
       <c r="N181" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -10685,7 +10685,7 @@
         <v>0.72</v>
       </c>
       <c r="K182" t="n">
-        <v>34.84</v>
+        <v>30.25</v>
       </c>
       <c r="L182" t="n">
         <v>0</v>
@@ -10694,7 +10694,7 @@
         <v>1</v>
       </c>
       <c r="N182" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="183">
@@ -10745,7 +10745,7 @@
         <v>0.72</v>
       </c>
       <c r="K183" t="n">
-        <v>14.78</v>
+        <v>38.95</v>
       </c>
       <c r="L183" t="n">
         <v>0</v>
@@ -10754,7 +10754,7 @@
         <v>1</v>
       </c>
       <c r="N183" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="184">
@@ -10805,7 +10805,7 @@
         <v>0.72</v>
       </c>
       <c r="K184" t="n">
-        <v>23.19</v>
+        <v>17.86</v>
       </c>
       <c r="L184" t="n">
         <v>0</v>
@@ -10814,7 +10814,7 @@
         <v>1</v>
       </c>
       <c r="N184" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="185">
@@ -10865,7 +10865,7 @@
         <v>0.72</v>
       </c>
       <c r="K185" t="n">
-        <v>10.21</v>
+        <v>46.79</v>
       </c>
       <c r="L185" t="n">
         <v>0</v>
@@ -10874,7 +10874,7 @@
         <v>1</v>
       </c>
       <c r="N185" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="186">
@@ -10925,7 +10925,7 @@
         <v>0.72</v>
       </c>
       <c r="K186" t="n">
-        <v>40.69</v>
+        <v>33.59</v>
       </c>
       <c r="L186" t="n">
         <v>0</v>
@@ -10934,7 +10934,7 @@
         <v>1</v>
       </c>
       <c r="N186" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="187">
@@ -10985,7 +10985,7 @@
         <v>0.72</v>
       </c>
       <c r="K187" t="n">
-        <v>45.8</v>
+        <v>32.66</v>
       </c>
       <c r="L187" t="n">
         <v>0</v>
@@ -10994,7 +10994,7 @@
         <v>1</v>
       </c>
       <c r="N187" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -11114,7 +11114,7 @@
         <v>1</v>
       </c>
       <c r="N189" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="190">
@@ -11174,7 +11174,7 @@
         <v>1</v>
       </c>
       <c r="N190" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="191">
@@ -11225,7 +11225,7 @@
         <v>0.8</v>
       </c>
       <c r="K191" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L191" t="n">
         <v>0</v>
@@ -11234,7 +11234,7 @@
         <v>1</v>
       </c>
       <c r="N191" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="192">
@@ -11285,7 +11285,7 @@
         <v>0.8</v>
       </c>
       <c r="K192" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L192" t="n">
         <v>0</v>
@@ -11294,7 +11294,7 @@
         <v>1</v>
       </c>
       <c r="N192" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="193">
@@ -11345,7 +11345,7 @@
         <v>0.8</v>
       </c>
       <c r="K193" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L193" t="n">
         <v>0</v>
@@ -11354,7 +11354,7 @@
         <v>1</v>
       </c>
       <c r="N193" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="194">
@@ -11405,7 +11405,7 @@
         <v>0.8</v>
       </c>
       <c r="K194" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L194" t="n">
         <v>0</v>
@@ -11414,7 +11414,7 @@
         <v>1</v>
       </c>
       <c r="N194" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="195">
@@ -11474,7 +11474,7 @@
         <v>1</v>
       </c>
       <c r="N195" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="196">
@@ -11525,7 +11525,7 @@
         <v>0.8</v>
       </c>
       <c r="K196" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="L196" t="n">
         <v>0</v>
@@ -11585,7 +11585,7 @@
         <v>0.8</v>
       </c>
       <c r="K197" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="L197" t="n">
         <v>0</v>
@@ -11594,7 +11594,7 @@
         <v>1</v>
       </c>
       <c r="N197" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="198">
@@ -11774,7 +11774,7 @@
         <v>1</v>
       </c>
       <c r="N200" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="201">
@@ -11894,7 +11894,7 @@
         <v>1</v>
       </c>
       <c r="N202" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="203">
@@ -11954,7 +11954,7 @@
         <v>1</v>
       </c>
       <c r="N203" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="204">
@@ -12014,7 +12014,7 @@
         <v>1</v>
       </c>
       <c r="N204" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="205">
@@ -12074,7 +12074,7 @@
         <v>1</v>
       </c>
       <c r="N205" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="206">
@@ -12134,7 +12134,7 @@
         <v>1</v>
       </c>
       <c r="N206" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="207">
@@ -12254,7 +12254,7 @@
         <v>1</v>
       </c>
       <c r="N208" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="209">
@@ -12314,7 +12314,7 @@
         <v>1</v>
       </c>
       <c r="N209" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="210">
@@ -12374,7 +12374,7 @@
         <v>1</v>
       </c>
       <c r="N210" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="211">
@@ -12434,7 +12434,7 @@
         <v>1</v>
       </c>
       <c r="N211" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="212">
@@ -12494,7 +12494,7 @@
         <v>1</v>
       </c>
       <c r="N212" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="213">
@@ -12511,15 +12511,15 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>NO_CANDIDATE</t>
+          <t>LOW_SCORE</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>0</v>
+        <v>0.2149</v>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>No candidate within broad window and tolerance</t>
+          <t>Top score (0.21) below review threshold</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -12534,19 +12534,19 @@
       </c>
       <c r="I213" t="inlineStr"/>
       <c r="J213" t="n">
-        <v>0</v>
+        <v>0.2149</v>
       </c>
       <c r="K213" t="n">
-        <v>0</v>
+        <v>25.62</v>
       </c>
       <c r="L213" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M213" t="n">
         <v>1</v>
       </c>
       <c r="N213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="214">
@@ -12555,58 +12555,50 @@
           <t>ORD-1197</t>
         </is>
       </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>UTR500196</t>
-        </is>
-      </c>
+      <c r="B214" t="inlineStr"/>
       <c r="C214" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>UNMATCHED</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>NO_CANDIDATE</t>
         </is>
       </c>
       <c r="E214" t="n">
-        <v>0.3105</v>
+        <v>0</v>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>No candidate within broad window and tolerance</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>deterministic</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>groq/compound</t>
-        </is>
-      </c>
-      <c r="I214" t="inlineStr">
-        <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr"/>
       <c r="J214" t="n">
-        <v>0.3105</v>
+        <v>0</v>
       </c>
       <c r="K214" t="n">
-        <v>59.09</v>
+        <v>0</v>
       </c>
       <c r="L214" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M214" t="n">
         <v>1</v>
       </c>
       <c r="N214" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="215">
@@ -12615,41 +12607,49 @@
           <t>ORD-1198</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr"/>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>UTR500208</t>
+        </is>
+      </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>UNMATCHED</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>LOW_SCORE</t>
+          <t>AI_REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>0.198</v>
+        <v>0.258</v>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Top score (0.20) below review threshold</t>
+          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>deterministic</t>
+          <t>groq</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="I215" t="inlineStr"/>
+          <t>groq/compound</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+        </is>
+      </c>
       <c r="J215" t="n">
-        <v>0.198</v>
+        <v>0.258</v>
       </c>
       <c r="K215" t="n">
-        <v>162.29</v>
+        <v>25.24</v>
       </c>
       <c r="L215" t="n">
         <v>5</v>
@@ -12658,7 +12658,7 @@
         <v>1</v>
       </c>
       <c r="N215" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="216">
@@ -12675,15 +12675,15 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>NO_CANDIDATE</t>
+          <t>LOW_SCORE</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>No candidate within broad window and tolerance</t>
+          <t>Top score (0.24) below review threshold</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
@@ -12698,19 +12698,19 @@
       </c>
       <c r="I216" t="inlineStr"/>
       <c r="J216" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="K216" t="n">
-        <v>0</v>
+        <v>95.78</v>
       </c>
       <c r="L216" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M216" t="n">
         <v>1</v>
       </c>
       <c r="N216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -12783,11 +12783,11 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>0.294</v>
+        <v>0.26</v>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Top score (0.29) below review threshold</t>
+          <t>Top score (0.26) below review threshold</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -12802,19 +12802,19 @@
       </c>
       <c r="I218" t="inlineStr"/>
       <c r="J218" t="n">
-        <v>0.294</v>
+        <v>0.26</v>
       </c>
       <c r="K218" t="n">
-        <v>58.37</v>
+        <v>212.8</v>
       </c>
       <c r="L218" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M218" t="n">
         <v>1</v>
       </c>
       <c r="N218" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219">
@@ -12875,58 +12875,50 @@
           <t>ORD-1203</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>UTR500198</t>
-        </is>
-      </c>
+      <c r="B220" t="inlineStr"/>
       <c r="C220" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>UNMATCHED</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>NO_CANDIDATE</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>0.29</v>
+        <v>0</v>
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>No candidate within broad window and tolerance</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>groq</t>
+          <t>deterministic</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>groq/compound</t>
-        </is>
-      </c>
-      <c r="I220" t="inlineStr">
-        <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr"/>
       <c r="J220" t="n">
-        <v>0.29</v>
+        <v>0</v>
       </c>
       <c r="K220" t="n">
-        <v>6.36</v>
+        <v>0</v>
       </c>
       <c r="L220" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M220" t="n">
         <v>1</v>
       </c>
       <c r="N220" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221">
@@ -12937,7 +12929,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>UTR500198</t>
+          <t>UTR500159</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -12951,7 +12943,7 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>0.32</v>
+        <v>0.246</v>
       </c>
       <c r="F221" t="inlineStr">
         <is>
@@ -12974,19 +12966,19 @@
         </is>
       </c>
       <c r="J221" t="n">
-        <v>0.32</v>
+        <v>0.246</v>
       </c>
       <c r="K221" t="n">
-        <v>44.26</v>
+        <v>133.28</v>
       </c>
       <c r="L221" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M221" t="n">
         <v>1</v>
       </c>
       <c r="N221" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="222">
@@ -13003,15 +12995,15 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>NO_CANDIDATE</t>
+          <t>LOW_SCORE</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>0</v>
+        <v>0.3358</v>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>No candidate within broad window and tolerance</t>
+          <t>Top score (0.34) below review threshold</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -13026,19 +13018,19 @@
       </c>
       <c r="I222" t="inlineStr"/>
       <c r="J222" t="n">
-        <v>0</v>
+        <v>0.3358</v>
       </c>
       <c r="K222" t="n">
-        <v>0</v>
+        <v>27.45</v>
       </c>
       <c r="L222" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M222" t="n">
         <v>1</v>
       </c>
       <c r="N222" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="223">
@@ -13098,7 +13090,7 @@
         <v>1</v>
       </c>
       <c r="N223" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="224">
@@ -13158,7 +13150,7 @@
         <v>1</v>
       </c>
       <c r="N224" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="225">
@@ -13218,7 +13210,7 @@
         <v>1</v>
       </c>
       <c r="N225" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="226">
@@ -13278,7 +13270,7 @@
         <v>1</v>
       </c>
       <c r="N226" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="227">
@@ -14169,7 +14161,7 @@
       <c r="A244" t="inlineStr"/>
       <c r="B244" t="inlineStr">
         <is>
-          <t>UTR500200</t>
+          <t>UTR500196</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -14221,7 +14213,7 @@
       <c r="A245" t="inlineStr"/>
       <c r="B245" t="inlineStr">
         <is>
-          <t>UTR500202</t>
+          <t>UTR500198</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -14273,7 +14265,7 @@
       <c r="A246" t="inlineStr"/>
       <c r="B246" t="inlineStr">
         <is>
-          <t>UTR500204</t>
+          <t>UTR500200</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -14325,7 +14317,7 @@
       <c r="A247" t="inlineStr"/>
       <c r="B247" t="inlineStr">
         <is>
-          <t>UTR500206</t>
+          <t>UTR500202</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -14377,7 +14369,7 @@
       <c r="A248" t="inlineStr"/>
       <c r="B248" t="inlineStr">
         <is>
-          <t>UTR500208</t>
+          <t>UTR500204</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -14429,7 +14421,7 @@
       <c r="A249" t="inlineStr"/>
       <c r="B249" t="inlineStr">
         <is>
-          <t>UTR500210</t>
+          <t>UTR500206</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -14481,7 +14473,7 @@
       <c r="A250" t="inlineStr"/>
       <c r="B250" t="inlineStr">
         <is>
-          <t>UTR500211</t>
+          <t>UTR500210</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -14533,7 +14525,7 @@
       <c r="A251" t="inlineStr"/>
       <c r="B251" t="inlineStr">
         <is>
-          <t>UTR500212</t>
+          <t>UTR500211</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -14585,7 +14577,7 @@
       <c r="A252" t="inlineStr"/>
       <c r="B252" t="inlineStr">
         <is>
-          <t>UTR500213</t>
+          <t>UTR500212</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -14637,7 +14629,7 @@
       <c r="A253" t="inlineStr"/>
       <c r="B253" t="inlineStr">
         <is>
-          <t>UTR500214</t>
+          <t>UTR500213</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -14689,7 +14681,7 @@
       <c r="A254" t="inlineStr"/>
       <c r="B254" t="inlineStr">
         <is>
-          <t>UTR500215</t>
+          <t>UTR500214</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -14741,7 +14733,7 @@
       <c r="A255" t="inlineStr"/>
       <c r="B255" t="inlineStr">
         <is>
-          <t>UTR500216</t>
+          <t>UTR500215</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
@@ -14793,7 +14785,7 @@
       <c r="A256" t="inlineStr"/>
       <c r="B256" t="inlineStr">
         <is>
-          <t>UTR500217</t>
+          <t>UTR500216</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -14845,7 +14837,7 @@
       <c r="A257" t="inlineStr"/>
       <c r="B257" t="inlineStr">
         <is>
-          <t>UTR500218</t>
+          <t>UTR500217</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -14897,7 +14889,7 @@
       <c r="A258" t="inlineStr"/>
       <c r="B258" t="inlineStr">
         <is>
-          <t>UTR500219</t>
+          <t>UTR500218</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -14949,7 +14941,7 @@
       <c r="A259" t="inlineStr"/>
       <c r="B259" t="inlineStr">
         <is>
-          <t>UTR500220</t>
+          <t>UTR500219</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -14994,6 +14986,58 @@
         <v>1</v>
       </c>
       <c r="N259" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr"/>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>UTR500220</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>UNMATCHED</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>NO_MATCH</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>0</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>No matching ledger record found</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>deterministic</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr"/>
+      <c r="J260" t="n">
+        <v>0</v>
+      </c>
+      <c r="K260" t="n">
+        <v>0</v>
+      </c>
+      <c r="L260" t="n">
+        <v>0</v>
+      </c>
+      <c r="M260" t="n">
+        <v>1</v>
+      </c>
+      <c r="N260" t="n">
         <v>0</v>
       </c>
     </row>
@@ -15035,13 +15079,13 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.2311</v>
+        <v>0.2267</v>
       </c>
       <c r="B2" t="n">
         <v>0.7378</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2311</v>
+        <v>0.2267</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
phase-final: submission hardening and debug reliability
</commit_message>
<xml_diff>
--- a/data/reconciliation_results.xlsx
+++ b/data/reconciliation_results.xlsx
@@ -13166,12 +13166,12 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>MATCHED</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>AI_REVIEW_REQUIRED</t>
+          <t>AI_CONFIRMED_MATCH</t>
         </is>
       </c>
       <c r="E225" t="n">
@@ -13179,7 +13179,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>AI Review: AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>AI Confirmed: UTR500249 has the best score due to matching date, presence of order ID, and a reasonable fee explanation.</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -13194,7 +13194,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>AI error: Error code: 429 - {'error': {'message': 'Rate limit reached for model `groq/compound` in organization `org_01m1nyjryne9p8680zhbpw42gx` service tier `on_demand` on requests per day (RPD): Limit 250, Used 250, Requested 1. Please try again in 5m45.6s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'requests', 'code': 'rate_limit_exceeded'}}. Safe fallback to REVIEW.</t>
+          <t>UTR500249 has the best score due to matching date, presence of order ID, and a reasonable fee explanation.</t>
         </is>
       </c>
       <c r="J225" t="n">
@@ -13270,7 +13270,7 @@
         <v>1</v>
       </c>
       <c r="N226" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="227">
@@ -15079,7 +15079,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.2267</v>
+        <v>0.2222</v>
       </c>
       <c r="B2" t="n">
         <v>0.7378</v>
@@ -15088,7 +15088,7 @@
         <v>0.2267</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.0196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>